<commit_message>
feat: daesun task_list를 kyungnam 형식으로 계정·실행여부 작성
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal_analyzer/daesun/task_list_daesun.xlsx
+++ b/journal_analyzer/daesun/task_list_daesun.xlsx
@@ -479,11 +479,11 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>45658</v>
+        <v>46023</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD 형식 (분개장 샘플의 회계일자 2025/01/01 기준 추정 — 실제 회계기간 확인 필요)</t>
+          <t>YYYY-MM-DD 형식</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46022</v>
+        <v>46387</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
   </sheetData>
@@ -518,13 +518,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>계정과목</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>정기예금</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>특정금전신탁</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>미지급금</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>미지급비용(기타)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>미지급비용(신용카드)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>미지급비용(지급이자)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>외상매입금</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>외상매출금</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>외주가공비(제)</t>
         </is>
       </c>
     </row>
@@ -539,40 +609,125 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>작업명</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>계정과목</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>거래처명</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>금액열</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
+          <t>※ 사용법: 작업명(자유기재) / 계정과목·거래처명은 콤마로 여러 개 가능 / 금액열: 차변·대변·both / 실행여부 Y인 행만 처리됨</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>※ 사용법: 작업명(자유기재) / 계정과목·거래처명은 콤마로 여러 개 가능 / 금액열: 차변·대변·both / 실행여부 Y인 행만 처리됨</t>
+          <t>작업명</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>계정과목</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>거래처명</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>금액열</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>분석01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>분석02</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>분석03</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>분석04</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>분석05</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -587,7 +742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -599,6 +754,162 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>구분</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>기타보증금</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>임대보증금</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>미지급금</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>미지급비용(기타)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>미지급비용(지급이자)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>미지급비용(신용카드)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>예수금(소득세)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>예수금(지방소득세)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>예수금(건강보험)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>예수금(고용보험)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>예수금(국민연금)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>부가세예수금</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>선수금</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>부채</t>
         </is>
       </c>
     </row>
@@ -613,7 +924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -625,6 +936,474 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>계정과목</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>건물</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>건물감가상각누계액</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>구축물</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>구축물감가상각누계액</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>기계장치</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>기계장치감가상각누계액</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>공구와기구감가상각누계액</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>차량운반구</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>차량운반구감가상각누계액</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>기타무형자산</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>기타보증금</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>임대보증금</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>미지급금</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>미지급비용(기타)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>미지급비용(신용카드)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>미지급비용(지급이자)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>예수금(소득세)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>예수금(지방소득세)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>예수금(건강보험)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>예수금(고용보험)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>예수금(국민연금)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>부가세예수금</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>선수금</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>퇴직급여충당금</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>퇴직연금미지급금</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>퇴직연금운용자산</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>퇴직급여(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>퇴직급여(판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>급료(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>임금(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>직원급료(판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>임원보수(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>임원보수(판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>제수당및상여금(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>제수당및상여금(판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>잡급(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>잡급(판)</t>
         </is>
       </c>
     </row>
@@ -639,13 +1418,97 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>계정과목</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>지급이자</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>원맥대연불이자</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>단기차입금</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>외화단기차입금</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>당좌차월</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>장기차입금</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>유동성장기부채</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>유동성장기차입금</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>전환사채</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>유동성전환사채</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>전환상환우선주</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>유동성전환상환우선주</t>
         </is>
       </c>
     </row>
@@ -660,7 +1523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -677,6 +1540,414 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>실행여부</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>건물</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>구축물</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>기계장치</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>차량운반구</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>기타무형자산</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>건물</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>구축물</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>기계장치</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>차량운반구</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>기타무형자산</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>기타보증금</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>기타보증금</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>임대보증금</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>임대보증금</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>퇴직급여충당금</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>퇴직급여충당금</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>퇴직연금운용자산</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>퇴직연금운용자산</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>퇴직연금미지급금</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>퇴직연금미지급금</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -691,7 +1962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -703,6 +1974,42 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>실행여부</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>지급임차료</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>지급수수료</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>차량유지비</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -717,28 +2024,145 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>구분: 차변(비용/손실), 대변(수익/이익), both(양쪽 합계) | 실행여부 Y인 행만 처리</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>계정과목</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>실행여부</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>손익구분</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>매출원가</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>매출원가</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>판매비와관리비</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>판관비</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>영업외수익</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>영업외수익</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>영업외비용</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>영업외비용</t>
         </is>
       </c>
     </row>
@@ -753,7 +2177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -765,6 +2189,18 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>실행여부</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>보통예금</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -779,7 +2215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -806,6 +2242,138 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>감가상각비(제)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>감가상각비(판)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>무형자산상각비(판)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>외화환산손실</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>외화환산이익</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>통화선도거래이익</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
         </is>
       </c>
     </row>
@@ -1534,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1571,6 +3139,158 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>건물</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>건물감가상각누계액</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>구축물</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>구축물감가상각누계액</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>기계장치</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>기계장치감가상각누계액</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>공구와기구감가상각누계액</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>차량운반구</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>차량운반구감가상각누계액</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>건물,구축물,기계장치,공구와기구</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
         </is>
       </c>
     </row>
@@ -1585,7 +3305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1607,6 +3327,23 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>유형자산처분이익</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>유형자산처분손실</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1672,13 +3409,16 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
+      </c>
+      <c r="F2" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -1697,7 +3437,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1822,7 +3562,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1872,7 +3612,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1947,7 +3687,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1972,7 +3712,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2122,7 +3862,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2147,7 +3887,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2172,7 +3912,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2197,7 +3937,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2222,7 +3962,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2247,7 +3987,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2272,7 +4012,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2297,7 +4037,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2317,7 +4057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2339,6 +4079,74 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>상품매출</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>제품매출</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>원재료</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>외주가공비(제)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -2353,7 +4161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2375,6 +4183,164 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>외상매출금</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>선급금</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>외주가공비(제)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>외상매입금</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>보통예금</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>보통예금</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>상품매출</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>제품매출</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>(전체)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>전체 계정 — 데이터 많을 경우 느릴 수 있음</t>
         </is>
       </c>
     </row>
@@ -2389,7 +4355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2416,6 +4382,138 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>외상매출금</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>외상매출금 상대계정</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>미수금</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>미수금 상대계정</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>보통예금</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>보통예금 상대계정</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>미지급금</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>미지급금 상대계정</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>제품매출</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>제품매출 상대계정</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>상품매출</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>상품매출 상대계정</t>
         </is>
       </c>
     </row>
@@ -2430,7 +4528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2476,7 +4574,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2501,7 +4599,32 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>보통예금</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>보통예금만 5억원 기준 (선택)</t>
         </is>
       </c>
     </row>
@@ -2542,7 +4665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2557,6 +4680,90 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>상품매출</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>제품매출</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>접대비(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>접대비(판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>접대비(판)경조</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>지급수수료(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>지급수수료(판)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: daesun task_list에 15_감사샘플링 시트 추가
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal_analyzer/daesun/task_list_daesun.xlsx
+++ b/journal_analyzer/daesun/task_list_daesun.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-19298" yWindow="-98" windowWidth="19396" windowHeight="12196" tabRatio="600" firstSheet="6" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,38 +16,59 @@
     <sheet name="11_특수관계자 분석" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="13_매출 vs 비용 교차" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="14_심층분석 (계정별 Top) " sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="17_거래처분석" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="20_잔액증감분석 (계정별 거래처별)" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="21_총계정원장" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="22_은행조회서 완전성" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="23_계정별 상세거래내역" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="24_리스완전성" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="25_손익월별분석" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="26_AI계정별분석_실행" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="27_감가상각_평가손익분석" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="감가상각_유형자산롤포워드" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="유형자산_처분손익" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="15_감사샘플링" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="17_거래처분석" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="20_잔액증감분석 (계정별 거래처별)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="21_총계정원장" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="22_은행조회서 완전성" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="23_계정별 상세거래내역" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="24_리스완전성" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="25_손익월별분석" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="26_AI계정별분석_실행" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="27_감가상각_평가손익분석" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="감가상각_유형자산롤포워드" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="유형자산_처분손익" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="4">
     <font>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <sz val="8"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -68,17 +88,27 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="쉼표 [0]" xfId="1" builtinId="6"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -442,7 +472,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -479,7 +509,7 @@
           <t>StartDate</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="5" t="n">
         <v>46023</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -494,7 +524,7 @@
           <t>EndDate</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="5" t="n">
         <v>46387</v>
       </c>
     </row>
@@ -519,8 +549,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -532,21 +562,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CMA</t>
+          <t>미수금</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>정기예금</t>
+          <t>미수수익</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>특정금전신탁</t>
+          <t>외상매입금</t>
         </is>
       </c>
     </row>
@@ -560,42 +590,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>미지급비용(기타)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>미지급비용(신용카드)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>미지급비용(지급이자)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>외상매입금</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>외상매출금</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>외주가공비(제)</t>
+          <t>미지급비용</t>
         </is>
       </c>
     </row>
@@ -610,129 +605,480 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>※ 사용법: 작업명(자유기재) / 계정과목·거래처명은 콤마로 여러 개 가능 / 금액열: 차변·대변·both / 실행여부 Y인 행만 처리됨</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>계정과목</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>시작일</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>종료일</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>샘플링방법</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>금액타입</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>샘플크기</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>통계표사용</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>신뢰수준</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>허용왜곡표시</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>예상왜곡표시</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>이상거래포함</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>개별유의금액</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>비고</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>작업명</t>
+          <t>외상매출금</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>계정과목</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>거래처명</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>금액열</t>
-        </is>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="n"/>
+      <c r="D2" s="8" t="n"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>실행여부</t>
+          <t>MUS</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J2" s="9" t="n"/>
+      <c r="K2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="n"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>예시) 매출 실재성 — 차변 MUS 30건</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>분석01</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
+          <t>보통예금</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
       <c r="E3" t="inlineStr">
         <is>
+          <t>체계적</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>40</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J3" s="9" t="n"/>
+      <c r="K3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="n"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>예시) 출금 증빙 — 대변 체계적 40건</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>분석02</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
+          <t>비품</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
       <c r="E4" t="inlineStr">
         <is>
+          <t>MUS</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
+      <c r="M4" s="9" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>예시) 통계표로 크기 계산 + 1천만원 이상 전수</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>분석03</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>분석04</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>분석05</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+    </row>
+    <row r="27">
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+    </row>
+    <row r="33">
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="8" t="n"/>
+    </row>
+    <row r="36">
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+    </row>
+    <row r="37">
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+    </row>
+    <row r="38">
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="8" t="n"/>
+    </row>
+    <row r="39">
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="8" t="n"/>
+    </row>
+    <row r="40">
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="C45" s="8" t="n"/>
+      <c r="D45" s="8" t="n"/>
+    </row>
+    <row r="46">
+      <c r="C46" s="8" t="n"/>
+      <c r="D46" s="8" t="n"/>
+    </row>
+    <row r="47">
+      <c r="C47" s="8" t="n"/>
+      <c r="D47" s="8" t="n"/>
+    </row>
+    <row r="48">
+      <c r="C48" s="8" t="n"/>
+      <c r="D48" s="8" t="n"/>
+    </row>
+    <row r="49">
+      <c r="C49" s="8" t="n"/>
+      <c r="D49" s="8" t="n"/>
+    </row>
+    <row r="50">
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+    </row>
+    <row r="51">
+      <c r="C51" s="8" t="n"/>
+      <c r="D51" s="8" t="n"/>
+    </row>
+    <row r="52">
+      <c r="C52" s="8" t="n"/>
+      <c r="D52" s="8" t="n"/>
+    </row>
+    <row r="53">
+      <c r="C53" s="8" t="n"/>
+      <c r="D53" s="8" t="n"/>
+    </row>
+    <row r="54">
+      <c r="C54" s="8" t="n"/>
+      <c r="D54" s="8" t="n"/>
+    </row>
+    <row r="55">
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+    </row>
+    <row r="56">
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="8" t="n"/>
+    </row>
+    <row r="57">
+      <c r="C57" s="8" t="n"/>
+      <c r="D57" s="8" t="n"/>
+    </row>
+    <row r="58">
+      <c r="C58" s="8" t="n"/>
+      <c r="D58" s="8" t="n"/>
+    </row>
+    <row r="59">
+      <c r="C59" s="8" t="n"/>
+      <c r="D59" s="8" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"MUS,체계적,무작위,금액상위"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"차변,대변,both"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B200 H2:H200 L2:L200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -743,174 +1089,139 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="10.4140625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="20.58203125" bestFit="1" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>계정명</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>구분</t>
+          <t>※ 사용법: 작업명(자유기재) / 계정과목·거래처명은 콤마로 여러 개 가능 / 금액열: 차변·대변·both / 실행여부 Y인 행만 처리됨</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>기타보증금</t>
+          <t>작업명</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>계정과목</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>거래처명</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>금액열</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>실행여부</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>임대보증금</t>
+          <t>분석01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>부채</t>
+          <t>단기대여금</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>박상정, 박관회, 박우정</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>미지급금</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>부채</t>
+          <t>분석02</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>미지급비용(기타)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>부채</t>
+          <t>분석03</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>미지급비용(지급이자)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>부채</t>
+          <t>분석04</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>미지급비용(신용카드)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>예수금(소득세)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>예수금(지방소득세)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>예수금(건강보험)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>예수금(고용보험)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>예수금(국민연금)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>부가세예수금</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>선수금</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>부채</t>
+          <t>분석05</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -925,486 +1236,174 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>계정명</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>구분</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>계정과목</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>기타보증금</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>자산</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>건물</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>임대보증금</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>건물감가상각누계액</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>미지급금</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>건설중인자산</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>미지급비용(기타)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>구축물</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>미지급비용(지급이자)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>구축물감가상각누계액</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>미지급비용(신용카드)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>기계장치</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>예수금(소득세)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>기계장치감가상각누계액</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>예수금(지방소득세)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>공구와기구</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>예수금(건강보험)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>공구와기구감가상각누계액</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>예수금(고용보험)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>차량운반구</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>예수금(국민연금)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>차량운반구감가상각누계액</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>부가세예수금</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>기타무형자산</t>
+          <t>부채</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>자산</t>
+          <t>선수금</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>기타보증금</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
           <t>부채</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>임대보증금</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>미지급금</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>미지급비용(기타)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>미지급비용(신용카드)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>미지급비용(지급이자)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>예수금(소득세)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>예수금(지방소득세)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>예수금(건강보험)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>예수금(고용보험)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>예수금(국민연금)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>부가세예수금</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>선수금</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>퇴직급여충당금</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>퇴직연금미지급금</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>부채</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>퇴직연금운용자산</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>퇴직급여(제)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>퇴직급여(판)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>급료(제)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>임금(제)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>직원급료(판)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>임원보수(제)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>임원보수(판)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>제수당및상여금(제)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>제수당및상여금(판)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>잡급(제)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>비용</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>잡급(판)</t>
         </is>
       </c>
     </row>
@@ -1419,12 +1418,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>계정과목</t>
         </is>
       </c>
@@ -1432,84 +1436,468 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>지급이자</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>건물</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>원맥대연불이자</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>건물감가상각누계액</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>단기차입금</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>외화단기차입금</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>구축물</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>당좌차월</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>구축물감가상각누계액</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>장기차입금</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>기계장치</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>유동성장기부채</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>기계장치감가상각누계액</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>유동성장기차입금</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>전환사채</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>공구와기구감가상각누계액</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>유동성전환사채</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>차량운반구</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>전환상환우선주</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>차량운반구감가상각누계액</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>유동성전환상환우선주</t>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>기타무형자산</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>자산</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>기타보증금</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>임대보증금</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>미지급금</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>미지급비용(기타)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>미지급비용(신용카드)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>미지급비용(지급이자)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>예수금(소득세)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>예수금(지방소득세)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>예수금(건강보험)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>예수금(고용보험)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>예수금(국민연금)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>부가세예수금</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>선수금</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>퇴직급여충당금</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>퇴직연금미지급금</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>부채</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>퇴직연금운용자산</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>퇴직급여(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>퇴직급여(판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>급료(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>임금(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>직원급료(판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>임원보수(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>임원보수(판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>제수당및상여금(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>제수당및상여금(판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>잡급(제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>비용</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>잡급(판)</t>
         </is>
       </c>
     </row>
@@ -1524,8 +1912,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="20.25" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1533,422 +1924,74 @@
           <t>계정과목</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>금액유형</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>건물</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>단기차입금</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>구축물</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>외화단기차입금</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>기계장치</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>당좌차월</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>공구와기구</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>장기차입금</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>차량운반구</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>유동성장기부채</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>건설중인자산</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>유동성장기차입금</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>기타무형자산</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>지급이자</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>건물</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>원맥대연불이자</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>구축물</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Y</t>
+          <t>지급수수료(판)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>기계장치</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>공구와기구</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>차량운반구</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>건설중인자산</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>기타무형자산</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>기타보증금</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>기타보증금</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>임대보증금</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>임대보증금</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>퇴직급여충당금</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>퇴직급여충당금</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
           <t>퇴직연금운용자산</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>퇴직연금운용자산</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>퇴직연금미지급금</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>퇴직연금미지급금</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1963,8 +2006,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="16.25" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1974,6 +2020,11 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>금액유형</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>실행여부</t>
         </is>
       </c>
@@ -1981,10 +2032,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>지급임차료</t>
+          <t>건물</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1993,10 +2049,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>지급수수료</t>
+          <t>구축물</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2005,10 +2066,372 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>차량유지비</t>
+          <t>기계장치</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>차량운반구</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>기타무형자산</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>건물</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>구축물</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>기계장치</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>차량운반구</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>기타무형자산</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>기타보증금</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>기타보증금</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>임대보증금</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>임대보증금</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>퇴직급여충당금</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>퇴직급여충당금</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>퇴직연금운용자산</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>퇴직연금운용자산</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>퇴직연금미지급금</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>퇴직연금미지급금</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2025,145 +2448,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>구분: 차변(비용/손실), 대변(수익/이익), both(양쪽 합계) | 실행여부 Y인 행만 처리</t>
+          <t>계정과목</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>실행여부</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>계정과목</t>
+          <t>지급임차료</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>실행여부</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>손익구분</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>매출</t>
+          <t>지급수수료</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>매출</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>매출원가</t>
+          <t>차량유지비</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>매출원가</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>판매비와관리비</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>판관비</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>영업외수익</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>영업외수익</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>영업외비용</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>영업외비용</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -2178,113 +2510,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="28.6640625" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>계정과목</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>샘플링비율</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>최소건수</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>최대건수</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>금액상위</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>최신</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>이상치</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>월별</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>랜덤</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>중점검토사항</t>
+          <t>구분: 차변(비용/손실), 대변(수익/이익), both(양쪽 합계) | 실행여부 Y인 행만 처리</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>보통예금</t>
+          <t>계정과목</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D2" t="n">
-        <v>30</v>
-      </c>
-      <c r="E2" t="n">
-        <v>150</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I2" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J2" s="3" t="n">
-        <v>0.1</v>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>손익구분</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>매출</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>매출원가</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>매출원가</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>판매비와관리비</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>판관비</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>영업외수익</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>영업외수익</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>영업외비용</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>영업외비용</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2298,8 +2666,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2309,154 +2687,211 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>금액열</t>
+          <t>실행여부</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>그룹기준열</t>
+          <t>샘플링비율</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>실행여부</t>
+          <t>최소건수</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>비고</t>
+          <t>최대건수</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>금액상위</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>최신</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>이상치</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>월별</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>랜덤</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>중점검토사항</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>감가상각비(제)</t>
+          <t>보통예금</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
-        </is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E2" t="n">
+        <v>150</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>감가상각비(판)</t>
+          <t>상품매출</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E3" t="n">
+        <v>150</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>분기말 매출 증가가 두드러지는 지 검토</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>무형자산상각비(판)</t>
+          <t>제품매출</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E4" t="n">
+        <v>150</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>분기말 매출 증가가 두드러지는 지 검토</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>외화환산손실</t>
+          <t>이자비용</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>외화환산이익</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>통화선도거래이익</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D5" t="n">
+        <v>30</v>
+      </c>
+      <c r="E5" t="n">
+        <v>150</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>월별 이자비용이 균등하게 발생하는 지 검토</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2907,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -2829,17 +3264,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AI계정별분석 (시트 미생성)</t>
+          <t>감사샘플링</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>계정과목 / 실행여부</t>
+          <t>계정과목 / 실행여부 / 시작일·종료일(선택) / 샘플링방법(MUS·체계적·무작위·금액상위) / 금액타입(차변·대변·both) / 샘플크기 / 통계표사용(Y/N) / 신뢰수준 / 허용왜곡표시 / 예상왜곡표시 / 이상거래포함(Y/N) / 개별유의금액(선택)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>쓰려면 시트명을 정확히 'AI계정별분석'으로 새로 만들고 계정과목 입력. Gemini 호출 없이 월별추이·샘플만 추출(26번과 형식은 같으나 AI 분석은 안 함)</t>
+          <t>계정 1줄 = 샘플링 1건, 샘플은 해당 계정의 전표 줄 단위(같은 전표의 상대계정 줄은 뽑지 않고 상대계정 열에 참고 표시). MUS=금액 누적 기준 구간마다 1건(구간보다 큰 줄은 반드시 선택) / 체계적=건수 기준 일정 간격 / 무작위 / 금액상위. 통계표사용=Y면 샘플크기 = 모집단금액×신뢰계수÷(허용왜곡표시−예상왜곡표시×확장계수) (95%: 3.0·1.6, 90%: 2.31·1.5). 이상거래포함=Y면 Z-score 3 이상·최대값을 샘플크기 안에서 우선 포함. 개별유의금액 이상은 샘플크기와 별도로 전수 포함. 시드 고정(42)이라 다시 돌려도 같은 샘플</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>결과: 샘플링조건(모집단·원장대사·크기근거·커버리지) + 계정별 샘플 시트(증빙종류·증빙확인·승인확인·예외사항·확인자 빈칸). AI로 보내지 않으므로 거래처·적요 실명 출력</t>
         </is>
       </c>
     </row>
@@ -3190,41 +3630,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="17.5" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>유형자산계정명</t>
+          <t>계정과목</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>감가상각누계액계정명</t>
+          <t>금액열</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>대체상대계정</t>
+          <t>그룹기준열</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>취득원가_수동조정</t>
+          <t>실행여부</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>상각누계액_수동조정</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -3233,152 +3666,132 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>건물</t>
+          <t>감가상각비(제)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>건물감가상각누계액</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>건설중인자산</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>구축물</t>
+          <t>감가상각비(판)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>구축물감가상각누계액</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>건설중인자산</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>기계장치</t>
+          <t>무형자산상각비(판)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>기계장치감가상각누계액</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>건설중인자산</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>공구와기구</t>
+          <t>외화환산손실</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>공구와기구감가상각누계액</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>건설중인자산</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>차량운반구</t>
+          <t>외화환산이익</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>차량운반구감가상각누계액</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>건설중인자산</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>건물,구축물,기계장치,공구와기구</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+          <t>통화선도거래이익</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>계정명/차대변 방향은 회사 실제 계정과목명에 맞게 조정 필요 (익/손 분리 계정이면 행 추가)</t>
         </is>
       </c>
     </row>
@@ -3393,8 +3806,215 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="14.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="24.1640625" bestFit="1" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>유형자산계정명</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>감가상각누계액계정명</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>대체상대계정</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>취득원가_수동조정</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>상각누계액_수동조정</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>건물</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>건물감가상각누계액</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>구축물</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>구축물감가상각누계액</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>기계장치</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>기계장치감가상각누계액</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>공구와기구감가상각누계액</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>차량운반구</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>차량운반구감가상각누계액</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>건설중인자산</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>건물,구축물,기계장치,공구와기구</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>daesun 분개장 계정명 기준 (2026-10-22) — 대체상대계정은 추정, 실행 후 확인 필요</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3447,7 +4067,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="8.5" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="28.83203125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="102" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="8.5" bestFit="1" customWidth="1" min="4" max="5"/>
+    <col width="6.6640625" bestFit="1" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3815,12 +4442,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AI 계정별 분석</t>
+          <t>감사샘플링</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>계정별 월별 추이 및 샘플 추출 → AI계정별분석 시트 참조</t>
+          <t>계정별 감사증빙 샘플 추출 (MUS/체계적/무작위/금액상위, 전표 줄 단위) → 15_감사샘플링 시트 참조</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3875,7 +4502,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3950,7 +4577,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -3975,7 +4602,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -4146,7 +4773,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="13.58203125" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4207,7 +4837,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>원재료</t>
+          <t>운반비(판)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4224,7 +4854,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>외주가공비(제)</t>
+          <t>지급수수료(판)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4249,8 +4879,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="13.58203125" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4294,12 +4927,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>선급금</t>
+          <t>외상매입금</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>차변</t>
+          <t>대변</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4311,7 +4944,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>외주가공비(제)</t>
+          <t>보통예금</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4328,7 +4961,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>외상매입금</t>
+          <t>보통예금</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4345,12 +4978,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>보통예금</t>
+          <t>상품매출</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>차변</t>
+          <t>대변</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4362,7 +4995,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>보통예금</t>
+          <t>제품매출</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4379,54 +5012,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>상품매출</t>
+          <t>(전체)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>대변</t>
+          <t>차변</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>제품매출</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>(전체)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>전체 계정 — 데이터 많을 경우 느릴 수 있음</t>
         </is>
@@ -4444,7 +5043,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="10.4140625" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4616,8 +5218,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <cols>
+    <col width="14.25" bestFit="1" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4657,7 +5262,7 @@
           <t>차변</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="6" t="n">
         <v>1000000000</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -4682,7 +5287,7 @@
           <t>대변</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="6" t="n">
         <v>1000000000</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -4702,7 +5307,7 @@
           <t>차변</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="6" t="n">
         <v>500000000</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -4713,6 +5318,46 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>보통예금만 5억원 기준 (선택)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>상품매출</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>500000001</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>제품매출</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>500000002</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -4728,7 +5373,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4754,7 +5399,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4771,7 +5416,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>매출</t>
+          <t>수익</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4783,7 +5428,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>매출</t>
+          <t>수익</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4812,7 +5457,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>접대비(판)</t>
+          <t>포장비(제)</t>
         </is>
       </c>
     </row>
@@ -4824,7 +5469,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>접대비(판)경조</t>
+          <t>운반비(판)</t>
         </is>
       </c>
     </row>
@@ -4836,7 +5481,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>지급수수료(제)</t>
+          <t>접대비(판)</t>
         </is>
       </c>
     </row>

</xml_diff>